<commit_message>
feat: hotel room number on the check-in form; drop address, map and event rooms
Attendees can enter the hotel room they stay in (optional, up to 20
characters). It is confirmed in the thank-you popup, shown and searchable in
the admin list, and exported as "Nomor Kamar Hotel". The Lokasi section
(address and map pin) is gone, so Leaflet is removed and the public page is
about 40 KB lighter, and the export no longer has address or coordinate
columns. The mock event-room list from the previous commit is removed.

Migration 20261028000000_guestbook_room_number_optional_address.sql adds
room_number and makes address optional. Until it is applied, the page checks
in the old way (no room, address "-") instead of failing.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/artifacts/contoh-ekspor-check-in.xlsx
+++ b/artifacts/contoh-ekspor-check-in.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K49"/>
+  <dimension ref="A1:I49"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -416,27 +416,21 @@
         <v>E-mail</v>
       </c>
       <c r="F1" t="str">
-        <v>Alamat</v>
+        <v>Nomor Kamar Hotel</v>
       </c>
       <c r="G1" t="str">
-        <v>Latitude</v>
+        <v>Berkas</v>
       </c>
       <c r="H1" t="str">
-        <v>Longitude</v>
+        <v>Hadiah</v>
       </c>
       <c r="I1" t="str">
-        <v>Berkas</v>
-      </c>
-      <c r="J1" t="str">
-        <v>Hadiah</v>
-      </c>
-      <c r="K1" t="str">
         <v>Waktu Undian (WIB)</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>26/10/2026 21:55 WIB</v>
+        <v>28/10/2026 12:49 WIB</v>
       </c>
       <c r="B2" t="str">
         <v/>
@@ -451,27 +445,21 @@
         <v>putri.santoso48@example.com</v>
       </c>
       <c r="F2" t="str">
-        <v>Jl. M.H. Thamrin No. 25, Jakarta Pusat</v>
+        <v/>
       </c>
       <c r="G2" t="str">
-        <v>-6.1742</v>
+        <v/>
       </c>
       <c r="H2" t="str">
-        <v>106.827</v>
+        <v/>
       </c>
       <c r="I2" t="str">
-        <v/>
-      </c>
-      <c r="J2" t="str">
-        <v/>
-      </c>
-      <c r="K2" t="str">
         <v/>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>26/10/2026 21:18 WIB</v>
+        <v>28/10/2026 12:12 WIB</v>
       </c>
       <c r="B3" t="str">
         <v/>
@@ -486,27 +474,21 @@
         <v>dimas.nugroho47@example.com</v>
       </c>
       <c r="F3" t="str">
-        <v>Jl. Jenderal Ahmad Yani No. 22, Makassar</v>
+        <v>1230</v>
       </c>
       <c r="G3" t="str">
-        <v>-5.1271</v>
+        <v/>
       </c>
       <c r="H3" t="str">
-        <v>119.4238</v>
+        <v/>
       </c>
       <c r="I3" t="str">
-        <v/>
-      </c>
-      <c r="J3" t="str">
-        <v/>
-      </c>
-      <c r="K3" t="str">
         <v/>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>26/10/2026 20:41 WIB</v>
+        <v>28/10/2026 11:35 WIB</v>
       </c>
       <c r="B4" t="str">
         <v/>
@@ -521,27 +503,21 @@
         <v>lestari.wijaya46@example.com</v>
       </c>
       <c r="F4" t="str">
-        <v>Jl. Asia Afrika No. 19, Bandung</v>
+        <v>1123</v>
       </c>
       <c r="G4" t="str">
-        <v>-6.9178</v>
+        <v/>
       </c>
       <c r="H4" t="str">
-        <v>107.603</v>
+        <v/>
       </c>
       <c r="I4" t="str">
-        <v/>
-      </c>
-      <c r="J4" t="str">
-        <v/>
-      </c>
-      <c r="K4" t="str">
         <v/>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>26/10/2026 20:04 WIB</v>
+        <v>28/10/2026 10:58 WIB</v>
       </c>
       <c r="B5" t="str">
         <v/>
@@ -556,27 +532,21 @@
         <v>bayu.siregar45@example.com</v>
       </c>
       <c r="F5" t="str">
-        <v>Jl. Teuku Umar No. 16, Denpasar</v>
+        <v>1016</v>
       </c>
       <c r="G5" t="str">
-        <v>-8.6788</v>
+        <v/>
       </c>
       <c r="H5" t="str">
-        <v>115.202</v>
+        <v/>
       </c>
       <c r="I5" t="str">
-        <v/>
-      </c>
-      <c r="J5" t="str">
-        <v/>
-      </c>
-      <c r="K5" t="str">
         <v/>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>26/10/2026 19:27 WIB</v>
+        <v>28/10/2026 10:21 WIB</v>
       </c>
       <c r="B6" t="str">
         <v/>
@@ -591,27 +561,21 @@
         <v>intan.hartono44@example.com</v>
       </c>
       <c r="F6" t="str">
-        <v>Jl. Gatot Subroto No. 13, Medan</v>
+        <v/>
       </c>
       <c r="G6" t="str">
-        <v>3.5857</v>
+        <v/>
       </c>
       <c r="H6" t="str">
-        <v>98.6702</v>
+        <v/>
       </c>
       <c r="I6" t="str">
-        <v/>
-      </c>
-      <c r="J6" t="str">
-        <v/>
-      </c>
-      <c r="K6" t="str">
         <v/>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>26/10/2026 18:50 WIB</v>
+        <v>28/10/2026 09:44 WIB</v>
       </c>
       <c r="B7" t="str">
         <v/>
@@ -626,30 +590,24 @@
         <v>fajar.simanjuntak43@example.com</v>
       </c>
       <c r="F7" t="str">
-        <v>Jl. Jenderal Sudirman No. 10, Jakarta Selatan</v>
+        <v>802</v>
       </c>
       <c r="G7" t="str">
-        <v>-6.233</v>
+        <v/>
       </c>
       <c r="H7" t="str">
-        <v>106.806</v>
+        <v/>
       </c>
       <c r="I7" t="str">
-        <v/>
-      </c>
-      <c r="J7" t="str">
-        <v/>
-      </c>
-      <c r="K7" t="str">
         <v/>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>26/10/2026 18:13 WIB</v>
+        <v>28/10/2026 09:07 WIB</v>
       </c>
       <c r="B8" t="str">
-        <v>26/10/2026 20:13 WIB</v>
+        <v>28/10/2026 11:07 WIB</v>
       </c>
       <c r="C8" t="str">
         <v>Ratna Saputra</v>
@@ -661,27 +619,21 @@
         <v>ratna.saputra42@example.com</v>
       </c>
       <c r="F8" t="str">
-        <v>Jl. Malioboro No. 7, Yogyakarta</v>
+        <v>725</v>
       </c>
       <c r="G8" t="str">
-        <v>-7.8046</v>
+        <v/>
       </c>
       <c r="H8" t="str">
-        <v>110.3658</v>
+        <v/>
       </c>
       <c r="I8" t="str">
-        <v/>
-      </c>
-      <c r="J8" t="str">
-        <v/>
-      </c>
-      <c r="K8" t="str">
         <v/>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>26/10/2026 17:36 WIB</v>
+        <v>28/10/2026 08:30 WIB</v>
       </c>
       <c r="B9" t="str">
         <v/>
@@ -696,27 +648,21 @@
         <v>joko.rahmawati41@example.com</v>
       </c>
       <c r="F9" t="str">
-        <v>Jl. Tunjungan No. 4, Surabaya</v>
+        <v>618</v>
       </c>
       <c r="G9" t="str">
-        <v>-7.2455</v>
+        <v/>
       </c>
       <c r="H9" t="str">
-        <v>112.7341</v>
+        <v/>
       </c>
       <c r="I9" t="str">
-        <v/>
-      </c>
-      <c r="J9" t="str">
-        <v/>
-      </c>
-      <c r="K9" t="str">
         <v/>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>26/10/2026 16:59 WIB</v>
+        <v>28/10/2026 07:53 WIB</v>
       </c>
       <c r="B10" t="str">
         <v/>
@@ -731,27 +677,21 @@
         <v>wulan.wibowo40@example.com</v>
       </c>
       <c r="F10" t="str">
-        <v>Jl. M.H. Thamrin No. 1, Jakarta Pusat</v>
+        <v/>
       </c>
       <c r="G10" t="str">
-        <v>-6.1782</v>
+        <v/>
       </c>
       <c r="H10" t="str">
-        <v>106.815</v>
+        <v/>
       </c>
       <c r="I10" t="str">
-        <v/>
-      </c>
-      <c r="J10" t="str">
-        <v/>
-      </c>
-      <c r="K10" t="str">
         <v/>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>26/10/2026 16:22 WIB</v>
+        <v>28/10/2026 07:16 WIB</v>
       </c>
       <c r="B11" t="str">
         <v/>
@@ -766,30 +706,24 @@
         <v>hendra.kusuma39@example.com</v>
       </c>
       <c r="F11" t="str">
-        <v>Jl. Jenderal Ahmad Yani No. 118, Makassar</v>
+        <v>1204</v>
       </c>
       <c r="G11" t="str">
-        <v>-5.1311</v>
+        <v/>
       </c>
       <c r="H11" t="str">
-        <v>119.4318</v>
+        <v/>
       </c>
       <c r="I11" t="str">
-        <v/>
-      </c>
-      <c r="J11" t="str">
-        <v/>
-      </c>
-      <c r="K11" t="str">
         <v/>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>26/10/2026 15:45 WIB</v>
+        <v>28/10/2026 06:39 WIB</v>
       </c>
       <c r="B12" t="str">
-        <v>26/10/2026 19:45 WIB</v>
+        <v>28/10/2026 10:39 WIB</v>
       </c>
       <c r="C12" t="str">
         <v>Nina Hasibuan</v>
@@ -801,27 +735,21 @@
         <v>nina.hasibuan38@example.com</v>
       </c>
       <c r="F12" t="str">
-        <v>Jl. Asia Afrika No. 115, Bandung</v>
+        <v>1127</v>
       </c>
       <c r="G12" t="str">
-        <v>-6.9218</v>
+        <v/>
       </c>
       <c r="H12" t="str">
-        <v>107.611</v>
+        <v/>
       </c>
       <c r="I12" t="str">
-        <v/>
-      </c>
-      <c r="J12" t="str">
-        <v/>
-      </c>
-      <c r="K12" t="str">
         <v/>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>26/10/2026 15:08 WIB</v>
+        <v>28/10/2026 06:02 WIB</v>
       </c>
       <c r="B13" t="str">
         <v/>
@@ -836,30 +764,24 @@
         <v>rudi.pratiwi37@example.com</v>
       </c>
       <c r="F13" t="str">
-        <v>Jl. Teuku Umar No. 112, Denpasar</v>
+        <v>1020</v>
       </c>
       <c r="G13" t="str">
-        <v>-8.6828</v>
+        <v/>
       </c>
       <c r="H13" t="str">
-        <v>115.21</v>
+        <v/>
       </c>
       <c r="I13" t="str">
-        <v/>
-      </c>
-      <c r="J13" t="str">
-        <v/>
-      </c>
-      <c r="K13" t="str">
         <v/>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>26/10/2026 14:31 WIB</v>
+        <v>28/10/2026 05:25 WIB</v>
       </c>
       <c r="B14" t="str">
-        <v>26/10/2026 16:31 WIB</v>
+        <v>28/10/2026 07:25 WIB</v>
       </c>
       <c r="C14" t="str">
         <v>Dewi Santoso</v>
@@ -871,27 +793,21 @@
         <v>dewi.santoso36@example.com</v>
       </c>
       <c r="F14" t="str">
-        <v>Jl. Gatot Subroto No. 109, Medan</v>
+        <v/>
       </c>
       <c r="G14" t="str">
-        <v>3.5817</v>
+        <v/>
       </c>
       <c r="H14" t="str">
-        <v>98.6582</v>
+        <v/>
       </c>
       <c r="I14" t="str">
-        <v/>
-      </c>
-      <c r="J14" t="str">
-        <v/>
-      </c>
-      <c r="K14" t="str">
         <v/>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>26/10/2026 13:54 WIB</v>
+        <v>28/10/2026 04:48 WIB</v>
       </c>
       <c r="B15" t="str">
         <v/>
@@ -906,30 +822,24 @@
         <v>agus.nugroho35@example.com</v>
       </c>
       <c r="F15" t="str">
-        <v>Jl. Jenderal Sudirman No. 106, Jakarta Selatan</v>
+        <v>806</v>
       </c>
       <c r="G15" t="str">
-        <v>-6.237</v>
+        <v/>
       </c>
       <c r="H15" t="str">
-        <v>106.794</v>
+        <v>Hadiah 2: Jam tangan pintar</v>
       </c>
       <c r="I15" t="str">
-        <v/>
-      </c>
-      <c r="J15" t="str">
-        <v>Hadiah 2: Jam tangan pintar</v>
-      </c>
-      <c r="K15" t="str">
-        <v>26/10/2026 21:20 WIB</v>
+        <v>28/10/2026 12:14 WIB</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>26/10/2026 13:17 WIB</v>
+        <v>28/10/2026 04:11 WIB</v>
       </c>
       <c r="B16" t="str">
-        <v>26/10/2026 19:17 WIB</v>
+        <v>28/10/2026 10:11 WIB</v>
       </c>
       <c r="C16" t="str">
         <v>Siti Wijaya</v>
@@ -941,27 +851,21 @@
         <v>siti.wijaya34@example.com</v>
       </c>
       <c r="F16" t="str">
-        <v>Jl. Malioboro No. 103, Yogyakarta</v>
+        <v>729</v>
       </c>
       <c r="G16" t="str">
-        <v>-7.7806</v>
+        <v/>
       </c>
       <c r="H16" t="str">
-        <v>110.3738</v>
+        <v/>
       </c>
       <c r="I16" t="str">
-        <v/>
-      </c>
-      <c r="J16" t="str">
-        <v/>
-      </c>
-      <c r="K16" t="str">
         <v/>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>26/10/2026 12:40 WIB</v>
+        <v>28/10/2026 03:34 WIB</v>
       </c>
       <c r="B17" t="str">
         <v/>
@@ -976,30 +880,24 @@
         <v>budi.siregar33@example.com</v>
       </c>
       <c r="F17" t="str">
-        <v>Jl. Tunjungan No. 100, Surabaya</v>
+        <v>622</v>
       </c>
       <c r="G17" t="str">
-        <v>-7.2495</v>
+        <v/>
       </c>
       <c r="H17" t="str">
-        <v>112.7421</v>
+        <v/>
       </c>
       <c r="I17" t="str">
-        <v/>
-      </c>
-      <c r="J17" t="str">
-        <v/>
-      </c>
-      <c r="K17" t="str">
         <v/>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>26/10/2026 12:03 WIB</v>
+        <v>28/10/2026 02:57 WIB</v>
       </c>
       <c r="B18" t="str">
-        <v>26/10/2026 16:03 WIB</v>
+        <v>28/10/2026 06:57 WIB</v>
       </c>
       <c r="C18" t="str">
         <v>Putri Hartono</v>
@@ -1011,27 +909,21 @@
         <v>putri.hartono32@example.com</v>
       </c>
       <c r="F18" t="str">
-        <v>Jl. M.H. Thamrin No. 97, Jakarta Pusat</v>
+        <v/>
       </c>
       <c r="G18" t="str">
-        <v>-6.1822</v>
+        <v/>
       </c>
       <c r="H18" t="str">
-        <v>106.823</v>
+        <v/>
       </c>
       <c r="I18" t="str">
-        <v/>
-      </c>
-      <c r="J18" t="str">
-        <v/>
-      </c>
-      <c r="K18" t="str">
         <v/>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>26/10/2026 11:26 WIB</v>
+        <v>28/10/2026 02:20 WIB</v>
       </c>
       <c r="B19" t="str">
         <v/>
@@ -1046,30 +938,24 @@
         <v>dimas.simanjuntak31@example.com</v>
       </c>
       <c r="F19" t="str">
-        <v>Jl. Jenderal Ahmad Yani No. 94, Makassar</v>
+        <v>1208</v>
       </c>
       <c r="G19" t="str">
-        <v>-5.1351</v>
+        <v/>
       </c>
       <c r="H19" t="str">
-        <v>119.4198</v>
+        <v/>
       </c>
       <c r="I19" t="str">
-        <v/>
-      </c>
-      <c r="J19" t="str">
-        <v/>
-      </c>
-      <c r="K19" t="str">
         <v/>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>26/10/2026 10:49 WIB</v>
+        <v>28/10/2026 01:43 WIB</v>
       </c>
       <c r="B20" t="str">
-        <v>26/10/2026 12:49 WIB</v>
+        <v>28/10/2026 03:43 WIB</v>
       </c>
       <c r="C20" t="str">
         <v>Lestari Saputra</v>
@@ -1081,27 +967,21 @@
         <v>lestari.saputra30@example.com</v>
       </c>
       <c r="F20" t="str">
-        <v>Jl. Asia Afrika No. 91, Bandung</v>
+        <v>1101</v>
       </c>
       <c r="G20" t="str">
-        <v>-6.9258</v>
+        <v/>
       </c>
       <c r="H20" t="str">
-        <v>107.599</v>
+        <v/>
       </c>
       <c r="I20" t="str">
-        <v/>
-      </c>
-      <c r="J20" t="str">
-        <v/>
-      </c>
-      <c r="K20" t="str">
         <v/>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>26/10/2026 10:12 WIB</v>
+        <v>28/10/2026 01:06 WIB</v>
       </c>
       <c r="B21" t="str">
         <v/>
@@ -1116,30 +996,24 @@
         <v>bayu.rahmawati29@example.com</v>
       </c>
       <c r="F21" t="str">
-        <v>Jl. Teuku Umar No. 88, Denpasar</v>
+        <v>1024</v>
       </c>
       <c r="G21" t="str">
-        <v>-8.6868</v>
+        <v/>
       </c>
       <c r="H21" t="str">
-        <v>115.218</v>
+        <v/>
       </c>
       <c r="I21" t="str">
-        <v/>
-      </c>
-      <c r="J21" t="str">
-        <v/>
-      </c>
-      <c r="K21" t="str">
         <v/>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>26/10/2026 09:35 WIB</v>
+        <v>28/10/2026 00:29 WIB</v>
       </c>
       <c r="B22" t="str">
-        <v>26/10/2026 15:35 WIB</v>
+        <v>28/10/2026 06:29 WIB</v>
       </c>
       <c r="C22" t="str">
         <v>Intan Wibowo</v>
@@ -1151,27 +1025,21 @@
         <v>intan.wibowo28@example.com</v>
       </c>
       <c r="F22" t="str">
-        <v>Jl. Gatot Subroto No. 85, Medan</v>
+        <v/>
       </c>
       <c r="G22" t="str">
-        <v>3.5777</v>
+        <v/>
       </c>
       <c r="H22" t="str">
-        <v>98.6662</v>
+        <v/>
       </c>
       <c r="I22" t="str">
-        <v/>
-      </c>
-      <c r="J22" t="str">
-        <v/>
-      </c>
-      <c r="K22" t="str">
         <v/>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>26/10/2026 08:58 WIB</v>
+        <v>27/10/2026 23:52 WIB</v>
       </c>
       <c r="B23" t="str">
         <v/>
@@ -1186,30 +1054,24 @@
         <v>fajar.kusuma27@example.com</v>
       </c>
       <c r="F23" t="str">
-        <v>Jl. Jenderal Sudirman No. 82, Jakarta Selatan</v>
+        <v>810</v>
       </c>
       <c r="G23" t="str">
-        <v>-6.213</v>
+        <v/>
       </c>
       <c r="H23" t="str">
-        <v>106.802</v>
+        <v/>
       </c>
       <c r="I23" t="str">
-        <v/>
-      </c>
-      <c r="J23" t="str">
-        <v/>
-      </c>
-      <c r="K23" t="str">
         <v/>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>26/10/2026 08:21 WIB</v>
+        <v>27/10/2026 23:15 WIB</v>
       </c>
       <c r="B24" t="str">
-        <v>26/10/2026 12:21 WIB</v>
+        <v>28/10/2026 03:15 WIB</v>
       </c>
       <c r="C24" t="str">
         <v>Ratna Hasibuan</v>
@@ -1221,27 +1083,21 @@
         <v>ratna.hasibuan26@example.com</v>
       </c>
       <c r="F24" t="str">
-        <v>Jl. Malioboro No. 79, Yogyakarta</v>
+        <v>703</v>
       </c>
       <c r="G24" t="str">
-        <v>-7.7846</v>
+        <v/>
       </c>
       <c r="H24" t="str">
-        <v>110.3618</v>
+        <v/>
       </c>
       <c r="I24" t="str">
-        <v/>
-      </c>
-      <c r="J24" t="str">
-        <v/>
-      </c>
-      <c r="K24" t="str">
         <v/>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>26/10/2026 07:44 WIB</v>
+        <v>27/10/2026 22:38 WIB</v>
       </c>
       <c r="B25" t="str">
         <v/>
@@ -1256,30 +1112,24 @@
         <v>joko.pratiwi25@example.com</v>
       </c>
       <c r="F25" t="str">
-        <v>Jl. Tunjungan No. 76, Surabaya</v>
+        <v>626</v>
       </c>
       <c r="G25" t="str">
-        <v>-7.2535</v>
+        <v/>
       </c>
       <c r="H25" t="str">
-        <v>112.7301</v>
+        <v/>
       </c>
       <c r="I25" t="str">
-        <v/>
-      </c>
-      <c r="J25" t="str">
-        <v/>
-      </c>
-      <c r="K25" t="str">
         <v/>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>26/10/2026 07:07 WIB</v>
+        <v>27/10/2026 22:01 WIB</v>
       </c>
       <c r="B26" t="str">
-        <v>26/10/2026 09:07 WIB</v>
+        <v>28/10/2026 00:01 WIB</v>
       </c>
       <c r="C26" t="str">
         <v>Wulan Santoso</v>
@@ -1291,27 +1141,21 @@
         <v>wulan.santoso24@example.com</v>
       </c>
       <c r="F26" t="str">
-        <v>Jl. M.H. Thamrin No. 73, Jakarta Pusat</v>
+        <v/>
       </c>
       <c r="G26" t="str">
-        <v>-6.1862</v>
+        <v/>
       </c>
       <c r="H26" t="str">
-        <v>106.831</v>
+        <v/>
       </c>
       <c r="I26" t="str">
-        <v/>
-      </c>
-      <c r="J26" t="str">
-        <v/>
-      </c>
-      <c r="K26" t="str">
         <v/>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>26/10/2026 06:30 WIB</v>
+        <v>27/10/2026 21:24 WIB</v>
       </c>
       <c r="B27" t="str">
         <v/>
@@ -1326,30 +1170,24 @@
         <v>hendra.nugroho23@example.com</v>
       </c>
       <c r="F27" t="str">
-        <v>Jl. Jenderal Ahmad Yani No. 70, Makassar</v>
+        <v>1212</v>
       </c>
       <c r="G27" t="str">
-        <v>-5.1391</v>
+        <v/>
       </c>
       <c r="H27" t="str">
-        <v>119.4278</v>
+        <v/>
       </c>
       <c r="I27" t="str">
-        <v/>
-      </c>
-      <c r="J27" t="str">
-        <v/>
-      </c>
-      <c r="K27" t="str">
         <v/>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>26/10/2026 05:53 WIB</v>
+        <v>27/10/2026 20:47 WIB</v>
       </c>
       <c r="B28" t="str">
-        <v>26/10/2026 11:53 WIB</v>
+        <v>28/10/2026 02:47 WIB</v>
       </c>
       <c r="C28" t="str">
         <v>Nina Wijaya</v>
@@ -1361,27 +1199,21 @@
         <v>nina.wijaya22@example.com</v>
       </c>
       <c r="F28" t="str">
-        <v>Jl. Asia Afrika No. 67, Bandung</v>
+        <v>1105</v>
       </c>
       <c r="G28" t="str">
-        <v>-6.9298</v>
+        <v/>
       </c>
       <c r="H28" t="str">
-        <v>107.607</v>
+        <v/>
       </c>
       <c r="I28" t="str">
-        <v/>
-      </c>
-      <c r="J28" t="str">
-        <v/>
-      </c>
-      <c r="K28" t="str">
         <v/>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>26/10/2026 05:16 WIB</v>
+        <v>27/10/2026 20:10 WIB</v>
       </c>
       <c r="B29" t="str">
         <v/>
@@ -1396,30 +1228,24 @@
         <v>rudi.siregar21@example.com</v>
       </c>
       <c r="F29" t="str">
-        <v>Jl. Teuku Umar No. 64, Denpasar</v>
+        <v>1028</v>
       </c>
       <c r="G29" t="str">
-        <v>-8.6908</v>
+        <v/>
       </c>
       <c r="H29" t="str">
-        <v>115.206</v>
+        <v/>
       </c>
       <c r="I29" t="str">
-        <v/>
-      </c>
-      <c r="J29" t="str">
-        <v/>
-      </c>
-      <c r="K29" t="str">
         <v/>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>26/10/2026 04:39 WIB</v>
+        <v>27/10/2026 19:33 WIB</v>
       </c>
       <c r="B30" t="str">
-        <v>26/10/2026 08:39 WIB</v>
+        <v>27/10/2026 23:33 WIB</v>
       </c>
       <c r="C30" t="str">
         <v>Dewi Hartono</v>
@@ -1431,27 +1257,21 @@
         <v>dewi.hartono20@example.com</v>
       </c>
       <c r="F30" t="str">
-        <v>Jl. Gatot Subroto No. 61, Medan</v>
+        <v/>
       </c>
       <c r="G30" t="str">
-        <v>3.6017</v>
+        <v/>
       </c>
       <c r="H30" t="str">
-        <v>98.6542</v>
+        <v/>
       </c>
       <c r="I30" t="str">
-        <v/>
-      </c>
-      <c r="J30" t="str">
-        <v/>
-      </c>
-      <c r="K30" t="str">
         <v/>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>26/10/2026 04:02 WIB</v>
+        <v>27/10/2026 18:56 WIB</v>
       </c>
       <c r="B31" t="str">
         <v/>
@@ -1466,30 +1286,24 @@
         <v>agus.simanjuntak19@example.com</v>
       </c>
       <c r="F31" t="str">
-        <v>Jl. Jenderal Sudirman No. 58, Jakarta Selatan</v>
+        <v>814</v>
       </c>
       <c r="G31" t="str">
-        <v>-6.217</v>
+        <v/>
       </c>
       <c r="H31" t="str">
-        <v>106.81</v>
+        <v>Hadiah 3: Voucher belanja</v>
       </c>
       <c r="I31" t="str">
-        <v/>
-      </c>
-      <c r="J31" t="str">
-        <v>Hadiah 3: Voucher belanja</v>
-      </c>
-      <c r="K31" t="str">
-        <v>26/10/2026 21:00 WIB</v>
+        <v>28/10/2026 11:54 WIB</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>26/10/2026 03:25 WIB</v>
+        <v>27/10/2026 18:19 WIB</v>
       </c>
       <c r="B32" t="str">
-        <v>26/10/2026 05:25 WIB</v>
+        <v>27/10/2026 20:19 WIB</v>
       </c>
       <c r="C32" t="str">
         <v>Siti Saputra</v>
@@ -1501,27 +1315,21 @@
         <v>siti.saputra18@example.com</v>
       </c>
       <c r="F32" t="str">
-        <v>Jl. Malioboro No. 55, Yogyakarta</v>
+        <v>707</v>
       </c>
       <c r="G32" t="str">
-        <v>-7.7886</v>
+        <v/>
       </c>
       <c r="H32" t="str">
-        <v>110.3698</v>
+        <v/>
       </c>
       <c r="I32" t="str">
-        <v/>
-      </c>
-      <c r="J32" t="str">
-        <v/>
-      </c>
-      <c r="K32" t="str">
         <v/>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>26/10/2026 02:48 WIB</v>
+        <v>27/10/2026 17:42 WIB</v>
       </c>
       <c r="B33" t="str">
         <v/>
@@ -1536,30 +1344,24 @@
         <v>budi.rahmawati17@example.com</v>
       </c>
       <c r="F33" t="str">
-        <v>Jl. Tunjungan No. 52, Surabaya</v>
+        <v>630</v>
       </c>
       <c r="G33" t="str">
-        <v>-7.2575</v>
+        <v/>
       </c>
       <c r="H33" t="str">
-        <v>112.7381</v>
+        <v/>
       </c>
       <c r="I33" t="str">
-        <v/>
-      </c>
-      <c r="J33" t="str">
-        <v/>
-      </c>
-      <c r="K33" t="str">
         <v/>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>26/10/2026 02:11 WIB</v>
+        <v>27/10/2026 17:05 WIB</v>
       </c>
       <c r="B34" t="str">
-        <v>26/10/2026 08:11 WIB</v>
+        <v>27/10/2026 23:05 WIB</v>
       </c>
       <c r="C34" t="str">
         <v>Putri Wibowo</v>
@@ -1571,27 +1373,21 @@
         <v>putri.wibowo16@example.com</v>
       </c>
       <c r="F34" t="str">
-        <v>Jl. M.H. Thamrin No. 49, Jakarta Pusat</v>
+        <v/>
       </c>
       <c r="G34" t="str">
-        <v>-6.1902</v>
+        <v/>
       </c>
       <c r="H34" t="str">
-        <v>106.819</v>
+        <v/>
       </c>
       <c r="I34" t="str">
-        <v/>
-      </c>
-      <c r="J34" t="str">
-        <v/>
-      </c>
-      <c r="K34" t="str">
         <v/>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>26/10/2026 01:34 WIB</v>
+        <v>27/10/2026 16:28 WIB</v>
       </c>
       <c r="B35" t="str">
         <v/>
@@ -1606,30 +1402,24 @@
         <v>dimas.kusuma15@example.com</v>
       </c>
       <c r="F35" t="str">
-        <v>Jl. Jenderal Ahmad Yani No. 46, Makassar</v>
+        <v>1216</v>
       </c>
       <c r="G35" t="str">
-        <v>-5.1431</v>
+        <v/>
       </c>
       <c r="H35" t="str">
-        <v>119.4158</v>
+        <v/>
       </c>
       <c r="I35" t="str">
-        <v/>
-      </c>
-      <c r="J35" t="str">
-        <v/>
-      </c>
-      <c r="K35" t="str">
         <v/>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>26/10/2026 00:57 WIB</v>
+        <v>27/10/2026 15:51 WIB</v>
       </c>
       <c r="B36" t="str">
-        <v>26/10/2026 04:57 WIB</v>
+        <v>27/10/2026 19:51 WIB</v>
       </c>
       <c r="C36" t="str">
         <v>Lestari Hasibuan</v>
@@ -1641,27 +1431,21 @@
         <v>lestari.hasibuan14@example.com</v>
       </c>
       <c r="F36" t="str">
-        <v>Jl. Asia Afrika No. 43, Bandung</v>
+        <v>1109</v>
       </c>
       <c r="G36" t="str">
-        <v>-6.9338</v>
+        <v/>
       </c>
       <c r="H36" t="str">
-        <v>107.615</v>
+        <v/>
       </c>
       <c r="I36" t="str">
-        <v/>
-      </c>
-      <c r="J36" t="str">
-        <v/>
-      </c>
-      <c r="K36" t="str">
         <v/>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>26/10/2026 00:20 WIB</v>
+        <v>27/10/2026 15:14 WIB</v>
       </c>
       <c r="B37" t="str">
         <v/>
@@ -1676,30 +1460,24 @@
         <v>bayu.pratiwi13@example.com</v>
       </c>
       <c r="F37" t="str">
-        <v>Jl. Teuku Umar No. 40, Denpasar</v>
+        <v>1002</v>
       </c>
       <c r="G37" t="str">
-        <v>-8.6668</v>
+        <v/>
       </c>
       <c r="H37" t="str">
-        <v>115.214</v>
+        <v/>
       </c>
       <c r="I37" t="str">
-        <v/>
-      </c>
-      <c r="J37" t="str">
-        <v/>
-      </c>
-      <c r="K37" t="str">
         <v/>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>25/10/2026 23:43 WIB</v>
+        <v>27/10/2026 14:37 WIB</v>
       </c>
       <c r="B38" t="str">
-        <v>26/10/2026 01:43 WIB</v>
+        <v>27/10/2026 16:37 WIB</v>
       </c>
       <c r="C38" t="str">
         <v>Intan Santoso</v>
@@ -1711,27 +1489,21 @@
         <v>intan.santoso12@example.com</v>
       </c>
       <c r="F38" t="str">
-        <v>Jl. Gatot Subroto No. 37, Medan</v>
+        <v/>
       </c>
       <c r="G38" t="str">
-        <v>3.5977</v>
+        <v/>
       </c>
       <c r="H38" t="str">
-        <v>98.6622</v>
+        <v/>
       </c>
       <c r="I38" t="str">
-        <v/>
-      </c>
-      <c r="J38" t="str">
-        <v/>
-      </c>
-      <c r="K38" t="str">
         <v/>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>25/10/2026 23:06 WIB</v>
+        <v>27/10/2026 14:00 WIB</v>
       </c>
       <c r="B39" t="str">
         <v/>
@@ -1746,30 +1518,24 @@
         <v>fajar.nugroho11@example.com</v>
       </c>
       <c r="F39" t="str">
-        <v>Jl. Jenderal Sudirman No. 34, Jakarta Selatan</v>
+        <v>818</v>
       </c>
       <c r="G39" t="str">
-        <v>-6.221</v>
+        <v/>
       </c>
       <c r="H39" t="str">
-        <v>106.798</v>
+        <v/>
       </c>
       <c r="I39" t="str">
-        <v/>
-      </c>
-      <c r="J39" t="str">
-        <v/>
-      </c>
-      <c r="K39" t="str">
         <v/>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>25/10/2026 22:29 WIB</v>
+        <v>27/10/2026 13:23 WIB</v>
       </c>
       <c r="B40" t="str">
-        <v>26/10/2026 04:29 WIB</v>
+        <v>27/10/2026 19:23 WIB</v>
       </c>
       <c r="C40" t="str">
         <v>Ratna Wijaya</v>
@@ -1781,27 +1547,21 @@
         <v>ratna.wijaya10@example.com</v>
       </c>
       <c r="F40" t="str">
-        <v>Jl. Malioboro No. 31, Yogyakarta</v>
+        <v>711</v>
       </c>
       <c r="G40" t="str">
-        <v>-7.7926</v>
+        <v/>
       </c>
       <c r="H40" t="str">
-        <v>110.3578</v>
+        <v/>
       </c>
       <c r="I40" t="str">
-        <v/>
-      </c>
-      <c r="J40" t="str">
-        <v/>
-      </c>
-      <c r="K40" t="str">
         <v/>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>25/10/2026 21:52 WIB</v>
+        <v>27/10/2026 12:46 WIB</v>
       </c>
       <c r="B41" t="str">
         <v/>
@@ -1816,30 +1576,24 @@
         <v>joko.siregar9@example.com</v>
       </c>
       <c r="F41" t="str">
-        <v>Jl. Tunjungan No. 28, Surabaya</v>
+        <v>604</v>
       </c>
       <c r="G41" t="str">
-        <v>-7.2615</v>
+        <v/>
       </c>
       <c r="H41" t="str">
-        <v>112.7461</v>
+        <v/>
       </c>
       <c r="I41" t="str">
-        <v/>
-      </c>
-      <c r="J41" t="str">
-        <v/>
-      </c>
-      <c r="K41" t="str">
         <v/>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>25/10/2026 21:15 WIB</v>
+        <v>27/10/2026 12:09 WIB</v>
       </c>
       <c r="B42" t="str">
-        <v>26/10/2026 01:15 WIB</v>
+        <v>27/10/2026 16:09 WIB</v>
       </c>
       <c r="C42" t="str">
         <v>Wulan Hartono</v>
@@ -1851,27 +1605,21 @@
         <v>wulan.hartono8@example.com</v>
       </c>
       <c r="F42" t="str">
-        <v>Jl. M.H. Thamrin No. 25, Jakarta Pusat</v>
+        <v/>
       </c>
       <c r="G42" t="str">
-        <v>-6.1942</v>
+        <v/>
       </c>
       <c r="H42" t="str">
-        <v>106.827</v>
+        <v/>
       </c>
       <c r="I42" t="str">
-        <v/>
-      </c>
-      <c r="J42" t="str">
-        <v/>
-      </c>
-      <c r="K42" t="str">
         <v/>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>25/10/2026 20:38 WIB</v>
+        <v>27/10/2026 11:32 WIB</v>
       </c>
       <c r="B43" t="str">
         <v/>
@@ -1886,30 +1634,24 @@
         <v>hendra.simanjuntak7@example.com</v>
       </c>
       <c r="F43" t="str">
-        <v>Jl. Jenderal Ahmad Yani No. 22, Makassar</v>
+        <v>1220</v>
       </c>
       <c r="G43" t="str">
-        <v>-5.1471</v>
+        <v/>
       </c>
       <c r="H43" t="str">
-        <v>119.4238</v>
+        <v/>
       </c>
       <c r="I43" t="str">
-        <v/>
-      </c>
-      <c r="J43" t="str">
-        <v/>
-      </c>
-      <c r="K43" t="str">
         <v/>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>25/10/2026 20:01 WIB</v>
+        <v>27/10/2026 10:55 WIB</v>
       </c>
       <c r="B44" t="str">
-        <v>25/10/2026 22:01 WIB</v>
+        <v>27/10/2026 12:55 WIB</v>
       </c>
       <c r="C44" t="str">
         <v>Nina Saputra</v>
@@ -1921,27 +1663,21 @@
         <v>nina.saputra6@example.com</v>
       </c>
       <c r="F44" t="str">
-        <v>Jl. Asia Afrika No. 19, Bandung</v>
+        <v>1113</v>
       </c>
       <c r="G44" t="str">
-        <v>-6.9098</v>
+        <v/>
       </c>
       <c r="H44" t="str">
-        <v>107.603</v>
+        <v/>
       </c>
       <c r="I44" t="str">
-        <v/>
-      </c>
-      <c r="J44" t="str">
-        <v/>
-      </c>
-      <c r="K44" t="str">
         <v/>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>25/10/2026 19:24 WIB</v>
+        <v>27/10/2026 10:18 WIB</v>
       </c>
       <c r="B45" t="str">
         <v/>
@@ -1956,30 +1692,24 @@
         <v>rudi.rahmawati5@example.com</v>
       </c>
       <c r="F45" t="str">
-        <v>Jl. Teuku Umar No. 16, Denpasar</v>
+        <v>1006</v>
       </c>
       <c r="G45" t="str">
-        <v>-8.6708</v>
+        <v/>
       </c>
       <c r="H45" t="str">
-        <v>115.202</v>
+        <v/>
       </c>
       <c r="I45" t="str">
-        <v/>
-      </c>
-      <c r="J45" t="str">
-        <v/>
-      </c>
-      <c r="K45" t="str">
         <v/>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>25/10/2026 18:47 WIB</v>
+        <v>27/10/2026 09:41 WIB</v>
       </c>
       <c r="B46" t="str">
-        <v>26/10/2026 00:47 WIB</v>
+        <v>27/10/2026 15:41 WIB</v>
       </c>
       <c r="C46" t="str">
         <v>Dewi Wibowo</v>
@@ -1991,27 +1721,21 @@
         <v>dewi.wibowo4@example.com</v>
       </c>
       <c r="F46" t="str">
-        <v>Jl. Gatot Subroto No. 13, Medan</v>
+        <v/>
       </c>
       <c r="G46" t="str">
-        <v>3.5937</v>
+        <v/>
       </c>
       <c r="H46" t="str">
-        <v>98.6702</v>
+        <v/>
       </c>
       <c r="I46" t="str">
-        <v/>
-      </c>
-      <c r="J46" t="str">
-        <v/>
-      </c>
-      <c r="K46" t="str">
         <v/>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v>25/10/2026 18:10 WIB</v>
+        <v>27/10/2026 09:04 WIB</v>
       </c>
       <c r="B47" t="str">
         <v/>
@@ -2026,30 +1750,24 @@
         <v>agus.kusuma3@example.com</v>
       </c>
       <c r="F47" t="str">
-        <v>Jl. Jenderal Sudirman No. 10, Jakarta Selatan</v>
+        <v>822</v>
       </c>
       <c r="G47" t="str">
-        <v>-6.225</v>
+        <v/>
       </c>
       <c r="H47" t="str">
-        <v>106.806</v>
+        <v>Hadiah 1: Smartphone</v>
       </c>
       <c r="I47" t="str">
-        <v/>
-      </c>
-      <c r="J47" t="str">
-        <v>Hadiah 1: Smartphone</v>
-      </c>
-      <c r="K47" t="str">
-        <v>26/10/2026 21:40 WIB</v>
+        <v>28/10/2026 12:34 WIB</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>25/10/2026 17:33 WIB</v>
+        <v>27/10/2026 08:27 WIB</v>
       </c>
       <c r="B48" t="str">
-        <v>25/10/2026 21:33 WIB</v>
+        <v>27/10/2026 12:27 WIB</v>
       </c>
       <c r="C48" t="str">
         <v>Siti Hasibuan</v>
@@ -2061,27 +1779,21 @@
         <v>siti.hasibuan2@example.com</v>
       </c>
       <c r="F48" t="str">
-        <v>Jl. Malioboro No. 7, Yogyakarta</v>
+        <v>715</v>
       </c>
       <c r="G48" t="str">
-        <v>-7.7966</v>
+        <v/>
       </c>
       <c r="H48" t="str">
-        <v>110.3658</v>
+        <v/>
       </c>
       <c r="I48" t="str">
-        <v/>
-      </c>
-      <c r="J48" t="str">
-        <v/>
-      </c>
-      <c r="K48" t="str">
         <v/>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>25/10/2026 16:56 WIB</v>
+        <v>27/10/2026 07:50 WIB</v>
       </c>
       <c r="B49" t="str">
         <v/>
@@ -2096,27 +1808,21 @@
         <v>budi.pratiwi1@example.com</v>
       </c>
       <c r="F49" t="str">
-        <v>Jl. Tunjungan No. 4, Surabaya</v>
+        <v>608</v>
       </c>
       <c r="G49" t="str">
-        <v>-7.2655</v>
+        <v/>
       </c>
       <c r="H49" t="str">
-        <v>112.7341</v>
+        <v/>
       </c>
       <c r="I49" t="str">
-        <v/>
-      </c>
-      <c r="J49" t="str">
-        <v/>
-      </c>
-      <c r="K49" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:K49"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I49"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>